<commit_message>
feat(excel): right-align year columns — H toujours LTM, RATIOS LTM toujours rempli
- _build_year_col passe en alignement droite : H=plus recent, D=plus ancien
  * 4 ans -> E,F,G,H remplis (D vide) ; 3 ans -> F,G,H (D,E vides)
  * H est TOUJOURS la colonne LTM, quelle que soit la quantite de donnees
- D5-H5 : etiquettes d'annee ecrites directement comme valeurs statiques
  depuis excel_writer.py (ex: 2022, 2023, 2024, "2025 (LTM)")
  * Remplace les formules F128/G128/D117 du template (fragiles, left-align)
  * D132-H132 : helpers backup hors zone impression
- ltm_year = max(year_col_map) — simplifie (H toujours present)
- CLAUDE.md mis a jour : v4 alignement droite
- preview/MC.PA/MC.PA_financials.xlsx regenere et verifie

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/MC.PA/MC.PA_financials.xlsx
+++ b/preview/MC.PA/MC.PA_financials.xlsx
@@ -29,7 +29,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'COMPARABLES'!$A$1:$L$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'SCENARIOS'!$A$1:$I$55</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'DASHBOARD'!$A$1:$N$94</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'DASHBOARD 2'!$A$1:$P$107</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -2855,7 +2854,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -2990,7 +2989,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3050,7 +3049,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3393,7 +3392,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3455,7 +3454,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3493,7 +3492,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -3702,7 +3701,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3765,7 +3764,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3845,7 +3844,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -3985,7 +3984,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4043,7 +4042,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4119,7 +4118,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4340,7 +4339,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4398,7 +4397,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4436,7 +4435,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4507,7 +4506,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4762,7 +4761,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4820,7 +4819,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4858,7 +4857,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4929,7 +4928,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5184,7 +5183,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5242,7 +5241,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5280,7 +5279,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5415,7 +5414,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5463,7 +5462,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5544,7 +5543,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5813,7 +5812,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5949,7 +5948,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="fr-FR"/>
               </a:p>
@@ -6113,7 +6112,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="fr-FR"/>
               </a:p>
@@ -6230,7 +6229,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6280,7 +6279,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6366,7 +6365,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -6547,7 +6546,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="fr-FR"/>
               </a:p>
@@ -6665,7 +6664,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6724,7 +6723,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6787,7 +6786,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -7530,25 +7529,20 @@
           <t>UNIT</t>
         </is>
       </c>
-      <c r="D5" s="24">
-        <f>IF(1&gt;$F$128,"",IF(1=$G$128,VALUE($D$117)&amp;" (LTM)",VALUE($D$117)-($G$128-1)))</f>
-        <v/>
-      </c>
-      <c r="E5" s="24">
-        <f>IF(2&gt;$F$128,"",IF(2=$G$128,VALUE($D$117)&amp;" (LTM)",VALUE($D$117)-($G$128-2)))</f>
-        <v/>
-      </c>
-      <c r="F5" s="24">
-        <f>IF(3&gt;$F$128,"",IF(3=$G$128,VALUE($D$117)&amp;" (LTM)",VALUE($D$117)-($G$128-3)))</f>
-        <v/>
-      </c>
-      <c r="G5" s="24">
-        <f>IF(4&gt;$F$128,"",IF(4=$G$128,VALUE($D$117)&amp;" (LTM)",VALUE($D$117)-($G$128-4)))</f>
-        <v/>
-      </c>
-      <c r="H5" s="24">
-        <f>IF(5&gt;$F$128,"",IF(5=$G$128,VALUE($D$117)&amp;" (LTM)",VALUE($D$117)-($G$128-5)))</f>
-        <v/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
+        <is>
+          <t>2025 (LTM)</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -7601,19 +7595,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D9" s="266" t="n">
+      <c r="D9" s="266" t="n"/>
+      <c r="E9" s="266" t="n">
         <v>79183</v>
       </c>
-      <c r="E9" s="266" t="n">
+      <c r="F9" s="266" t="n">
         <v>86153</v>
       </c>
-      <c r="F9" s="266" t="n">
+      <c r="G9" s="266" t="n">
         <v>84682</v>
       </c>
-      <c r="G9" s="266" t="n">
+      <c r="H9" s="266" t="n">
         <v>80807</v>
       </c>
-      <c r="H9" s="266" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="3" t="n"/>
@@ -7627,19 +7621,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D10" s="267" t="n">
+      <c r="D10" s="267" t="n"/>
+      <c r="E10" s="267" t="n">
         <v>-24988</v>
       </c>
-      <c r="E10" s="267" t="n">
+      <c r="F10" s="267" t="n">
         <v>-26876</v>
       </c>
-      <c r="F10" s="267" t="n">
+      <c r="G10" s="267" t="n">
         <v>-27918</v>
       </c>
-      <c r="G10" s="267" t="n">
+      <c r="H10" s="267" t="n">
         <v>-27279</v>
       </c>
-      <c r="H10" s="267" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="3" t="n"/>
@@ -7721,19 +7715,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D14" s="266" t="n">
+      <c r="D14" s="266" t="n"/>
+      <c r="E14" s="266" t="n">
         <v>-33178</v>
       </c>
-      <c r="E14" s="266" t="n">
+      <c r="F14" s="266" t="n">
         <v>-36482</v>
       </c>
-      <c r="F14" s="266" t="n">
+      <c r="G14" s="266" t="n">
         <v>-37222</v>
       </c>
-      <c r="G14" s="266" t="n">
+      <c r="H14" s="266" t="n">
         <v>-35848</v>
       </c>
-      <c r="H14" s="266" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="3" t="n"/>
@@ -7765,19 +7759,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D16" s="268" t="n">
+      <c r="D16" s="268" t="n"/>
+      <c r="E16" s="268" t="n">
         <v>-6226</v>
       </c>
-      <c r="E16" s="268" t="n">
+      <c r="F16" s="268" t="n">
         <v>-7177</v>
       </c>
-      <c r="F16" s="268" t="n">
+      <c r="G16" s="268" t="n">
         <v>-7796</v>
       </c>
-      <c r="G16" s="268" t="n">
+      <c r="H16" s="268" t="n">
         <v>-8001</v>
       </c>
-      <c r="H16" s="268" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="3" t="n"/>
@@ -7859,19 +7853,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D20" s="266" t="n">
+      <c r="D20" s="266" t="n"/>
+      <c r="E20" s="266" t="n">
         <v>-382</v>
       </c>
-      <c r="E20" s="266" t="n">
+      <c r="F20" s="266" t="n">
         <v>-973</v>
       </c>
-      <c r="F20" s="266" t="n">
+      <c r="G20" s="266" t="n">
         <v>-1186</v>
       </c>
-      <c r="G20" s="266" t="n">
+      <c r="H20" s="266" t="n">
         <v>-1151</v>
       </c>
-      <c r="H20" s="266" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="3" t="n"/>
@@ -7885,19 +7879,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D21" s="268" t="n">
+      <c r="D21" s="268" t="n"/>
+      <c r="E21" s="268" t="n">
         <v>113</v>
       </c>
-      <c r="E21" s="268" t="n">
+      <c r="F21" s="268" t="n">
         <v>212</v>
       </c>
-      <c r="F21" s="268" t="n">
+      <c r="G21" s="268" t="n">
         <v>151</v>
       </c>
-      <c r="G21" s="268" t="n">
+      <c r="H21" s="268" t="n">
         <v>164</v>
       </c>
-      <c r="H21" s="268" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="3" t="n"/>
@@ -7979,19 +7973,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D25" s="266" t="n">
+      <c r="D25" s="266" t="n"/>
+      <c r="E25" s="266" t="n">
         <v>-5362</v>
       </c>
-      <c r="E25" s="266" t="n">
+      <c r="F25" s="266" t="n">
         <v>-5673</v>
       </c>
-      <c r="F25" s="266" t="n">
+      <c r="G25" s="266" t="n">
         <v>-5157</v>
       </c>
-      <c r="G25" s="266" t="n">
+      <c r="H25" s="266" t="n">
         <v>-5476</v>
       </c>
-      <c r="H25" s="266" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" thickBot="1">
       <c r="A26" s="3" t="n"/>
@@ -8142,19 +8136,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D34" s="269" t="n">
+      <c r="D34" s="269" t="n"/>
+      <c r="E34" s="269" t="n">
         <v>7300</v>
       </c>
-      <c r="E34" s="269" t="n">
+      <c r="F34" s="269" t="n">
         <v>7774</v>
       </c>
-      <c r="F34" s="269" t="n">
+      <c r="G34" s="269" t="n">
         <v>9631</v>
       </c>
-      <c r="G34" s="269" t="n">
+      <c r="H34" s="269" t="n">
         <v>8794</v>
       </c>
-      <c r="H34" s="269" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="3" t="n"/>
@@ -8168,19 +8162,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D35" s="266" t="n">
+      <c r="D35" s="266" t="n"/>
+      <c r="E35" s="266" t="n">
         <v>4258</v>
       </c>
-      <c r="E35" s="266" t="n">
+      <c r="F35" s="266" t="n">
         <v>4728</v>
       </c>
-      <c r="F35" s="266" t="n">
+      <c r="G35" s="266" t="n">
         <v>4731</v>
       </c>
-      <c r="G35" s="266" t="n">
+      <c r="H35" s="266" t="n">
         <v>4332</v>
       </c>
-      <c r="H35" s="266" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="3" t="n"/>
@@ -8194,19 +8188,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D36" s="266" t="n">
+      <c r="D36" s="266" t="n"/>
+      <c r="E36" s="266" t="n">
         <v>20319</v>
       </c>
-      <c r="E36" s="266" t="n">
+      <c r="F36" s="266" t="n">
         <v>22952</v>
       </c>
-      <c r="F36" s="266" t="n">
+      <c r="G36" s="266" t="n">
         <v>23669</v>
       </c>
-      <c r="G36" s="266" t="n">
+      <c r="H36" s="266" t="n">
         <v>22659</v>
       </c>
-      <c r="H36" s="266" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="3" t="n"/>
@@ -8220,17 +8214,17 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D37" s="268" t="n">
+      <c r="D37" s="268" t="n"/>
+      <c r="E37" s="268" t="n">
         <v>7488</v>
       </c>
-      <c r="E37" s="268" t="n"/>
-      <c r="F37" s="268" t="n">
-        <v>-1</v>
-      </c>
+      <c r="F37" s="268" t="n"/>
       <c r="G37" s="268" t="n">
         <v>-1</v>
       </c>
-      <c r="H37" s="268" t="n"/>
+      <c r="H37" s="268" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="3" t="n"/>
@@ -8297,19 +8291,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D41" s="266" t="n">
+      <c r="D41" s="266" t="n"/>
+      <c r="E41" s="266" t="n">
         <v>37670</v>
       </c>
-      <c r="E41" s="266" t="n">
+      <c r="F41" s="266" t="n">
         <v>42695</v>
       </c>
-      <c r="F41" s="266" t="n">
+      <c r="G41" s="266" t="n">
         <v>45895</v>
       </c>
-      <c r="G41" s="266" t="n">
+      <c r="H41" s="266" t="n">
         <v>44018</v>
       </c>
-      <c r="H41" s="266" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="3" t="n"/>
@@ -8323,19 +8317,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D42" s="266" t="n">
+      <c r="D42" s="266" t="n"/>
+      <c r="E42" s="266" t="n">
         <v>50214</v>
       </c>
-      <c r="E42" s="266" t="n">
+      <c r="F42" s="266" t="n">
         <v>49610</v>
       </c>
-      <c r="F42" s="266" t="n">
+      <c r="G42" s="266" t="n">
         <v>46880</v>
       </c>
-      <c r="G42" s="266" t="n">
+      <c r="H42" s="266" t="n">
         <v>41702</v>
       </c>
-      <c r="H42" s="266" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="3" t="n"/>
@@ -8349,19 +8343,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D43" s="266" t="n">
+      <c r="D43" s="266" t="n"/>
+      <c r="E43" s="266" t="n">
         <v>1186</v>
       </c>
-      <c r="E43" s="266" t="n">
+      <c r="F43" s="266" t="n">
         <v>99</v>
       </c>
-      <c r="F43" s="266" t="n">
+      <c r="G43" s="266" t="n">
         <v>127</v>
       </c>
-      <c r="G43" s="266" t="n">
+      <c r="H43" s="266" t="n">
         <v>128</v>
       </c>
-      <c r="H43" s="266" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
       <c r="A44" s="3" t="n"/>
@@ -8428,19 +8422,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D47" s="266" t="n">
+      <c r="D47" s="266" t="n"/>
+      <c r="E47" s="266" t="n">
         <v>8788</v>
       </c>
-      <c r="E47" s="266" t="n">
+      <c r="F47" s="266" t="n">
         <v>9049</v>
       </c>
-      <c r="F47" s="266" t="n">
+      <c r="G47" s="266" t="n">
         <v>8630</v>
       </c>
-      <c r="G47" s="266" t="n">
+      <c r="H47" s="266" t="n">
         <v>8223</v>
       </c>
-      <c r="H47" s="266" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="3" t="n"/>
@@ -8454,19 +8448,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D48" s="266" t="n">
+      <c r="D48" s="266" t="n"/>
+      <c r="E48" s="266" t="n">
         <v>9359</v>
       </c>
-      <c r="E48" s="266" t="n">
+      <c r="F48" s="266" t="n">
         <v>10680</v>
       </c>
-      <c r="F48" s="266" t="n">
+      <c r="G48" s="266" t="n">
         <v>10850</v>
       </c>
-      <c r="G48" s="266" t="n">
+      <c r="H48" s="266" t="n">
         <v>7925</v>
       </c>
-      <c r="H48" s="266" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="3" t="n"/>
@@ -8480,19 +8474,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D49" s="266" t="n">
+      <c r="D49" s="266" t="n"/>
+      <c r="E49" s="266" t="n">
         <v>1211</v>
       </c>
-      <c r="E49" s="266" t="n">
+      <c r="F49" s="266" t="n">
         <v>2541</v>
       </c>
-      <c r="F49" s="266" t="n">
+      <c r="G49" s="266" t="n">
         <v>2766</v>
       </c>
-      <c r="G49" s="266" t="n">
+      <c r="H49" s="266" t="n">
         <v>2123</v>
       </c>
-      <c r="H49" s="266" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="3" t="n"/>
@@ -8506,19 +8500,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D50" s="268" t="n">
+      <c r="D50" s="268" t="n"/>
+      <c r="E50" s="268" t="n">
         <v>9553</v>
       </c>
-      <c r="E50" s="268" t="n">
+      <c r="F50" s="268" t="n">
         <v>1880</v>
       </c>
-      <c r="F50" s="268" t="n">
+      <c r="G50" s="268" t="n">
         <v>1978</v>
       </c>
-      <c r="G50" s="268" t="n">
+      <c r="H50" s="268" t="n">
         <v>1910</v>
       </c>
-      <c r="H50" s="268" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="3" t="n"/>
@@ -8585,19 +8579,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D54" s="268" t="n">
+      <c r="D54" s="268" t="n"/>
+      <c r="E54" s="268" t="n">
         <v>10380</v>
       </c>
-      <c r="E54" s="268" t="n">
+      <c r="F54" s="268" t="n">
         <v>11227</v>
       </c>
-      <c r="F54" s="268" t="n">
+      <c r="G54" s="268" t="n">
         <v>12091</v>
       </c>
-      <c r="G54" s="268" t="n">
+      <c r="H54" s="268" t="n">
         <v>12419</v>
       </c>
-      <c r="H54" s="268" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="3" t="n"/>
@@ -8664,19 +8658,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D58" s="266" t="n">
+      <c r="D58" s="266" t="n"/>
+      <c r="E58" s="266" t="n">
         <v>1440</v>
       </c>
-      <c r="E58" s="266" t="n">
+      <c r="F58" s="266" t="n">
         <v>681</v>
       </c>
-      <c r="F58" s="266" t="n">
+      <c r="G58" s="266" t="n">
         <v>203</v>
       </c>
-      <c r="G58" s="266" t="n">
+      <c r="H58" s="266" t="n">
         <v>149</v>
       </c>
-      <c r="H58" s="266" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="3" t="n"/>
@@ -8914,19 +8908,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D71" s="266" t="n">
+      <c r="D71" s="266" t="n"/>
+      <c r="E71" s="266" t="n">
         <v>-394</v>
       </c>
-      <c r="E71" s="266" t="n">
+      <c r="F71" s="266" t="n">
         <v>-695</v>
       </c>
-      <c r="F71" s="266" t="n">
+      <c r="G71" s="266" t="n">
         <v>137</v>
       </c>
-      <c r="G71" s="266" t="n">
+      <c r="H71" s="266" t="n">
         <v>213</v>
       </c>
-      <c r="H71" s="266" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="3" t="n"/>
@@ -8940,19 +8934,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D72" s="266" t="n">
+      <c r="D72" s="266" t="n"/>
+      <c r="E72" s="266" t="n">
         <v>-4169</v>
       </c>
-      <c r="E72" s="266" t="n">
+      <c r="F72" s="266" t="n">
         <v>-4230</v>
       </c>
-      <c r="F72" s="266" t="n">
+      <c r="G72" s="266" t="n">
         <v>-1114</v>
       </c>
-      <c r="G72" s="266" t="n">
+      <c r="H72" s="266" t="n">
         <v>-1315</v>
       </c>
-      <c r="H72" s="266" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="3" t="n"/>
@@ -8966,19 +8960,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D73" s="266" t="n">
+      <c r="D73" s="266" t="n"/>
+      <c r="E73" s="266" t="n">
         <v>1532</v>
       </c>
-      <c r="E73" s="266" t="n">
+      <c r="F73" s="266" t="n">
         <v>434</v>
       </c>
-      <c r="F73" s="266" t="n">
+      <c r="G73" s="266" t="n">
         <v>-664</v>
       </c>
-      <c r="G73" s="266" t="n">
+      <c r="H73" s="266" t="n">
         <v>215</v>
       </c>
-      <c r="H73" s="266" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="3" t="n"/>
@@ -8992,19 +8986,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D74" s="266" t="n">
+      <c r="D74" s="266" t="n"/>
+      <c r="E74" s="266" t="n">
         <v>-483</v>
       </c>
-      <c r="E74" s="266" t="n">
+      <c r="F74" s="266" t="n">
         <v>-259</v>
       </c>
-      <c r="F74" s="266" t="n">
+      <c r="G74" s="266" t="n">
         <v>488</v>
       </c>
-      <c r="G74" s="266" t="n">
+      <c r="H74" s="266" t="n">
         <v>-172</v>
       </c>
-      <c r="H74" s="266" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" thickBot="1">
       <c r="A75" s="3" t="n"/>
@@ -9071,19 +9065,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D78" s="266" t="n">
+      <c r="D78" s="266" t="n"/>
+      <c r="E78" s="266" t="n">
         <v>-5082</v>
       </c>
-      <c r="E78" s="266" t="n">
+      <c r="F78" s="266" t="n">
         <v>-7807</v>
       </c>
-      <c r="F78" s="266" t="n">
+      <c r="G78" s="266" t="n">
         <v>-5552</v>
       </c>
-      <c r="G78" s="266" t="n">
+      <c r="H78" s="266" t="n">
         <v>-4670</v>
       </c>
-      <c r="H78" s="266" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="3" t="n"/>
@@ -9168,19 +9162,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D83" s="266" t="n">
+      <c r="D83" s="266" t="n"/>
+      <c r="E83" s="266" t="n">
         <v>3774</v>
       </c>
-      <c r="E83" s="266" t="n">
+      <c r="F83" s="266" t="n">
         <v>5990</v>
       </c>
-      <c r="F83" s="266" t="n">
+      <c r="G83" s="266" t="n">
         <v>3595</v>
       </c>
-      <c r="G83" s="266" t="n">
+      <c r="H83" s="266" t="n">
         <v>2095</v>
       </c>
-      <c r="H83" s="266" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="3" t="n"/>
@@ -9194,19 +9188,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D84" s="266" t="n">
-        <v>0</v>
-      </c>
+      <c r="D84" s="266" t="n"/>
       <c r="E84" s="266" t="n">
         <v>0</v>
       </c>
       <c r="F84" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="266" t="n">
         <v>53</v>
       </c>
-      <c r="G84" s="266" t="n">
+      <c r="H84" s="266" t="n">
         <v>0</v>
       </c>
-      <c r="H84" s="266" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="3" t="n"/>
@@ -9220,19 +9214,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D85" s="266" t="n">
+      <c r="D85" s="266" t="n"/>
+      <c r="E85" s="266" t="n">
         <v>-1616</v>
       </c>
-      <c r="E85" s="266" t="n">
+      <c r="F85" s="266" t="n">
         <v>-1584</v>
       </c>
-      <c r="F85" s="266" t="n">
+      <c r="G85" s="266" t="n">
         <v>-312</v>
       </c>
-      <c r="G85" s="266" t="n">
+      <c r="H85" s="266" t="n">
         <v>-1640</v>
       </c>
-      <c r="H85" s="266" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" thickBot="1">
       <c r="A86" s="3" t="n"/>
@@ -9332,19 +9326,19 @@
           <t>($000)</t>
         </is>
       </c>
-      <c r="D90" s="266" t="n">
+      <c r="D90" s="266" t="n"/>
+      <c r="E90" s="266" t="n">
         <v>7817</v>
       </c>
-      <c r="E90" s="266" t="n">
+      <c r="F90" s="266" t="n">
         <v>7100</v>
       </c>
-      <c r="F90" s="266" t="n">
+      <c r="G90" s="266" t="n">
         <v>7520</v>
       </c>
-      <c r="G90" s="266" t="n">
+      <c r="H90" s="266" t="n">
         <v>9269</v>
       </c>
-      <c r="H90" s="266" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1" thickBot="1">
       <c r="A91" s="3" t="n"/>
@@ -9430,7 +9424,7 @@
       <c r="F95" s="266" t="n"/>
       <c r="G95" s="266" t="n"/>
       <c r="H95" s="266" t="n">
-        <v>458.8</v>
+        <v>460.95</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -9556,7 +9550,7 @@
       <c r="F100" s="266" t="n"/>
       <c r="G100" s="266" t="n"/>
       <c r="H100" s="266" t="n">
-        <v>0.0433</v>
+        <v>0.0437</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -9692,7 +9686,7 @@
       <c r="F106" s="266" t="n"/>
       <c r="G106" s="266" t="n"/>
       <c r="H106" s="266" t="n">
-        <v>0.9179</v>
+        <v>0.9183</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
@@ -9712,7 +9706,7 @@
       <c r="F107" s="266" t="n"/>
       <c r="G107" s="266" t="n"/>
       <c r="H107" s="266" t="n">
-        <v>0.08210000000000001</v>
+        <v>0.08169999999999999</v>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1">
@@ -9901,7 +9895,7 @@
         </is>
       </c>
       <c r="D117" s="95" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E117" s="46" t="n"/>
       <c r="F117" s="46" t="n"/>
@@ -10084,11 +10078,11 @@
       </c>
       <c r="E128" s="419" t="n"/>
       <c r="F128" s="419">
-        <f>IF(D9&lt;&gt;"",1,0)+IF(E9&lt;&gt;"",1,0)+IF(F9&lt;&gt;"",1,0)+IF(G9&lt;&gt;"",1,0)+IF(H9&lt;&gt;"",1,0)</f>
+        <f>IF(COUNTA(D9,D10,D14,D15,D16,D20,D21,D25)=8,1,0)+IF(COUNTA(E9,E10,E14,E15,E16,E20,E21,E25)=8,1,0)+IF(COUNTA(F9,F10,F14,F15,F16,F20,F21,F25)=8,1,0)+IF(COUNTA(G9,G10,G14,G15,G16,G20,G21,G25)=8,1,0)+IF(COUNTA(H9,H10,H14,H15,H16,H20,H21,H25)=8,1,0)</f>
         <v/>
       </c>
       <c r="G128" s="419">
-        <f>IF(NOT(ISBLANK(H9)),F128,IF(NOT(ISBLANK(G9)),F128,IF(NOT(ISBLANK(F9)),F128,IF(NOT(ISBLANK(E9)),F128,IF(NOT(ISBLANK(D9)),F128,0)))))</f>
+        <f>IF(COUNTA(H9,H10,H14,H15,H16,H20,H21,H25)=8,$F$128,IF(COUNTA(G9,G10,G14,G15,G16,G20,G21,G25)=8,$F$128,IF(COUNTA(F9,F10,F14,F15,F16,F20,F21,F25)=8,$F$128,IF(COUNTA(E9,E10,E14,E15,E16,E20,E21,E25)=8,$F$128,IF(COUNTA(D9,D10,D14,D15,D16,D20,D21,D25)=8,$F$128,0)))))</f>
         <v/>
       </c>
       <c r="H128" s="419" t="n"/>
@@ -10108,7 +10102,7 @@
       <c r="B130" s="51" t="n"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>LVMH affiche une résilience remarquable malgré un environnement macroéconomique difficile. La marque maintient des marges exceptionnelles et une croissance organique solide dans le luxe.</t>
+          <t>LVMH affiche une résilience exceptionnelle malgré un environnement macroéconomique difficile, avec des marges maintenues à des niveaux records. La marque reste un leader incontesté du luxe, avec une c</t>
         </is>
       </c>
     </row>
@@ -10116,12 +10110,24 @@
       <c r="B131" s="51" t="n"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Invalidation : Ralentissement Chine &gt; -5% PIB ou perte LV Chine &gt; 3% ou concurrence Hermès accrue</t>
+          <t>Invalidation : Ralentissement Chine &gt; -5% PIB ou perte de parts de marché &gt;5% en Chine</t>
         </is>
       </c>
     </row>
     <row r="132" ht="15" customHeight="1">
       <c r="B132" s="51" t="n"/>
+      <c r="E132" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F132" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G132" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H132" t="n">
+        <v>2025</v>
+      </c>
     </row>
     <row r="133" ht="15" customHeight="1">
       <c r="B133" s="51" t="n"/>
@@ -10213,7 +10219,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.005555555555555556" right="0.005555555555555556" top="0.006944444444444444" bottom="0.006944444444444444" header="0.002777777777777778" footer="0.002777777777777778"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="73" fitToHeight="0"/>
 </worksheet>
 </file>
 
@@ -10411,7 +10417,7 @@
         </is>
       </c>
       <c r="C14" s="536" t="n">
-        <v>458.8</v>
+        <v>460.95</v>
       </c>
     </row>
     <row r="15">
@@ -16691,7 +16697,7 @@
         <v/>
       </c>
       <c r="H9" s="440">
-        <f>IF(INPUT!H9&lt;&gt;"",INPUT!H9,INPUT!G9)</f>
+        <f>INPUT!H9</f>
         <v/>
       </c>
       <c r="I9" s="441">
@@ -16741,7 +16747,7 @@
         <v/>
       </c>
       <c r="H10" s="445">
-        <f>IF(INPUT!H10&lt;&gt;"",INPUT!H10,INPUT!G10)</f>
+        <f>INPUT!H10</f>
         <v/>
       </c>
       <c r="I10" s="445">
@@ -16857,7 +16863,7 @@
         <v/>
       </c>
       <c r="H13" s="441">
-        <f>IF(INPUT!H14&lt;&gt;"",INPUT!H14,INPUT!G14)</f>
+        <f>INPUT!H14</f>
         <v/>
       </c>
       <c r="I13" s="441">
@@ -16907,7 +16913,7 @@
         <v/>
       </c>
       <c r="H14" s="445">
-        <f>IF(INPUT!H15&lt;&gt;"",INPUT!H15,INPUT!G15)</f>
+        <f>INPUT!H15</f>
         <v/>
       </c>
       <c r="I14" s="445">
@@ -16957,7 +16963,7 @@
         <v/>
       </c>
       <c r="H15" s="431">
-        <f>IF(INPUT!H30&lt;&gt;"",INPUT!H30,INPUT!G30)</f>
+        <f>INPUT!H30</f>
         <v/>
       </c>
       <c r="I15" s="431">
@@ -17023,7 +17029,7 @@
         <v/>
       </c>
       <c r="H17" s="445">
-        <f>IF(INPUT!H16&lt;&gt;"",INPUT!H16,INPUT!G16)</f>
+        <f>INPUT!H16</f>
         <v/>
       </c>
       <c r="I17" s="445">
@@ -17139,7 +17145,7 @@
         <v/>
       </c>
       <c r="H20" s="445">
-        <f>IF(INPUT!H20&lt;&gt;"",INPUT!H20,INPUT!G20)</f>
+        <f>INPUT!H20</f>
         <v/>
       </c>
       <c r="I20" s="445">
@@ -17255,7 +17261,7 @@
         <v/>
       </c>
       <c r="H23" s="441">
-        <f>IF(INPUT!H24&lt;&gt;"",INPUT!H24,INPUT!G24)</f>
+        <f>INPUT!H24</f>
         <v/>
       </c>
       <c r="I23" s="441">
@@ -17438,7 +17444,7 @@
       </c>
       <c r="C29" s="9" t="n"/>
       <c r="D29" s="457">
-        <f>IFERROR(IF(NOT(ISBLANK(INPUT!H9)),INPUT!H9/INPUT!G9-1,IF(NOT(ISBLANK(INPUT!G9)),INPUT!G9/INPUT!F9-1,IF(NOT(ISBLANK(INPUT!F9)),INPUT!F9/INPUT!E9-1,IF(NOT(ISBLANK(INPUT!E9)),INPUT!E9/INPUT!D9-1,0.05)))),0.05)</f>
+        <f>IFERROR(INPUT!H9/INPUT!G9-1,0.05)</f>
         <v/>
       </c>
       <c r="E29" s="458">
@@ -17452,7 +17458,7 @@
       <c r="G29" s="459" t="n"/>
       <c r="H29" s="459" t="n"/>
       <c r="I29" s="457">
-        <f>IFERROR(IF(NOT(ISBLANK(INPUT!H9)),INPUT!H9/INPUT!G9-1,IF(NOT(ISBLANK(INPUT!G9)),INPUT!G9/INPUT!F9-1,IF(NOT(ISBLANK(INPUT!F9)),INPUT!F9/INPUT!E9-1,IF(NOT(ISBLANK(INPUT!E9)),INPUT!E9/INPUT!D9-1,0.05)))),0.05)</f>
+        <f>IFERROR(INPUT!H9/INPUT!G9-1,0.05)</f>
         <v/>
       </c>
       <c r="J29" s="460">
@@ -18114,7 +18120,7 @@
         <v/>
       </c>
       <c r="H47" s="441">
-        <f>IF(INPUT!H78&lt;&gt;"",INPUT!H78,INPUT!G78)</f>
+        <f>INPUT!H78</f>
         <v/>
       </c>
       <c r="I47" s="441">
@@ -18164,7 +18170,7 @@
         <v/>
       </c>
       <c r="H48" s="441">
-        <f>IF(INPUT!H70&lt;&gt;"",INPUT!H70,INPUT!G70)+IF(INPUT!H71&lt;&gt;"",INPUT!H71,INPUT!G71)+IF(INPUT!H72&lt;&gt;"",INPUT!H72,INPUT!G72)+IF(INPUT!H73&lt;&gt;"",INPUT!H73,INPUT!G73)</f>
+        <f>INPUT!H70+INPUT!H71+INPUT!H72+INPUT!H73</f>
         <v/>
       </c>
       <c r="I48" s="441">
@@ -20306,7 +20312,7 @@
         </is>
       </c>
       <c r="D9" s="477" t="n">
-        <v>257.35</v>
+        <v>258.85</v>
       </c>
       <c r="E9" s="36" t="n">
         <v>45966.46</v>
@@ -20347,7 +20353,7 @@
         </is>
       </c>
       <c r="D10" s="477" t="n">
-        <v>353.2</v>
+        <v>353.15</v>
       </c>
       <c r="E10" s="36" t="n">
         <v>189993.22</v>
@@ -20388,7 +20394,7 @@
         </is>
       </c>
       <c r="D11" s="477" t="n">
-        <v>63.52</v>
+        <v>63.84</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>28259.39</v>
@@ -20429,7 +20435,7 @@
         </is>
       </c>
       <c r="D12" s="477" t="n">
-        <v>139.25</v>
+        <v>139.75</v>
       </c>
       <c r="E12" s="36" t="n">
         <v>80357.48</v>
@@ -21169,19 +21175,19 @@
         </is>
       </c>
       <c r="D37" s="485">
-        <f>INPUT!H95</f>
+        <f>INPUT!F95</f>
         <v/>
       </c>
       <c r="E37" s="485">
-        <f>INPUT!H95</f>
+        <f>INPUT!F95</f>
         <v/>
       </c>
       <c r="F37" s="485">
-        <f>INPUT!H95</f>
+        <f>INPUT!F95</f>
         <v/>
       </c>
       <c r="G37" s="485">
-        <f>INPUT!H95</f>
+        <f>INPUT!F95</f>
         <v/>
       </c>
       <c r="H37" s="22" t="n"/>
@@ -25811,7 +25817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD107"/>
+  <dimension ref="A1:AF107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="15.33203125" customWidth="1" style="167" min="1" max="1"/>
@@ -28379,7 +28385,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.005555555555555556" right="0.005555555555555556" top="0.005555555555555556" bottom="0.005555555555555556" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="10"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(excel): dynamisme complet colonnes annees + CF + F128 + COMPARABLES
- Conditional formatting inversee pour strategie right-align (H=LTM)
  D: <5, E: <4, F: <3, G: <2, H: <1 (etait D:<1...H:<5)
- F128 formule simplifiee: compte revenus non-vides (ex-COUNTA=8)
  corrects pour societes sans R&D (ex: MC.PA/LVMH)
- COMPARABLES share price: INPUT!F95 -> INPUT!H95 (colonne LTM)
- Page setup INPUT: portrait scale=82 (ex-fitToWidth qui ne fonctionnait pas)
- assets/TEMPLATE.xlsx mis a jour avec tous les correctifs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/preview/MC.PA/MC.PA_financials.xlsx
+++ b/preview/MC.PA/MC.PA_financials.xlsx
@@ -29,6 +29,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'COMPARABLES'!$A$1:$L$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'SCENARIOS'!$A$1:$I$55</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'DASHBOARD'!$A$1:$N$94</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'DASHBOARD 2'!$A$1:$P$107</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -2854,7 +2855,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -2989,7 +2990,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3049,7 +3050,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3392,7 +3393,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3454,7 +3455,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3492,7 +3493,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -3701,7 +3702,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3764,7 +3765,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -3844,7 +3845,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -3984,7 +3985,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4042,7 +4043,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4118,7 +4119,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4339,7 +4340,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4397,7 +4398,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4435,7 +4436,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4506,7 +4507,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4761,7 +4762,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4819,7 +4820,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -4857,7 +4858,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -4928,7 +4929,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5183,7 +5184,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5241,7 +5242,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5279,7 +5280,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5414,7 +5415,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5462,7 +5463,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -5543,7 +5544,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5812,7 +5813,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -5948,7 +5949,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="fr-FR"/>
               </a:p>
@@ -6112,7 +6113,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="fr-FR"/>
               </a:p>
@@ -6229,7 +6230,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6279,7 +6280,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6365,7 +6366,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="fr-FR"/>
         </a:p>
@@ -6546,7 +6547,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="fr-FR"/>
               </a:p>
@@ -6664,7 +6665,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6723,7 +6724,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -6786,7 +6787,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -10078,7 +10079,7 @@
       </c>
       <c r="E128" s="419" t="n"/>
       <c r="F128" s="419">
-        <f>IF(COUNTA(D9,D10,D14,D15,D16,D20,D21,D25)=8,1,0)+IF(COUNTA(E9,E10,E14,E15,E16,E20,E21,E25)=8,1,0)+IF(COUNTA(F9,F10,F14,F15,F16,F20,F21,F25)=8,1,0)+IF(COUNTA(G9,G10,G14,G15,G16,G20,G21,G25)=8,1,0)+IF(COUNTA(H9,H10,H14,H15,H16,H20,H21,H25)=8,1,0)</f>
+        <f>IF(D9&lt;&gt;"",1,0)+IF(E9&lt;&gt;"",1,0)+IF(F9&lt;&gt;"",1,0)+IF(G9&lt;&gt;"",1,0)+IF(H9&lt;&gt;"",1,0)</f>
         <v/>
       </c>
       <c r="G128" s="419">
@@ -10189,12 +10190,12 @@
   </sheetData>
   <conditionalFormatting sqref="D1:D122">
     <cfRule type="expression" priority="6" dxfId="0">
-      <formula>$F$128&lt;1</formula>
+      <formula>$F$128&lt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:E122">
     <cfRule type="expression" priority="7" dxfId="0">
-      <formula>$F$128&lt;2</formula>
+      <formula>$F$128&lt;4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F122">
@@ -10204,12 +10205,12 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G122">
     <cfRule type="expression" priority="9" dxfId="0">
-      <formula>$F$128&lt;4</formula>
+      <formula>$F$128&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:H122">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>$F$128&lt;5</formula>
+      <formula>$F$128&lt;1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -10219,7 +10220,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.005555555555555556" right="0.005555555555555556" top="0.006944444444444444" bottom="0.006944444444444444" header="0.002777777777777778" footer="0.002777777777777778"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="73" fitToHeight="0"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="82" fitToHeight="0"/>
 </worksheet>
 </file>
 
@@ -21175,19 +21176,19 @@
         </is>
       </c>
       <c r="D37" s="485">
-        <f>INPUT!F95</f>
+        <f>INPUT!H95</f>
         <v/>
       </c>
       <c r="E37" s="485">
-        <f>INPUT!F95</f>
+        <f>INPUT!H95</f>
         <v/>
       </c>
       <c r="F37" s="485">
-        <f>INPUT!F95</f>
+        <f>INPUT!H95</f>
         <v/>
       </c>
       <c r="G37" s="485">
-        <f>INPUT!F95</f>
+        <f>INPUT!H95</f>
         <v/>
       </c>
       <c r="H37" s="22" t="n"/>
@@ -25817,7 +25818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF107"/>
+  <dimension ref="A1:AD107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="15.33203125" customWidth="1" style="167" min="1" max="1"/>
@@ -28385,7 +28386,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.005555555555555556" right="0.005555555555555556" top="0.005555555555555556" bottom="0.005555555555555556" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" scale="10"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>